<commit_message>
started 2026.2.0-rc, added details queryPossibleMatches
</commit_message>
<xml_diff>
--- a/output/all-profiles.xlsx
+++ b/output/all-profiles.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12922" uniqueCount="1087">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13706" uniqueCount="1117">
   <si>
     <t>Property</t>
   </si>
@@ -36,7 +36,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2026.1.0</t>
+    <t>2026.2.0-rc</t>
   </si>
   <si>
     <t>Name</t>
@@ -3176,7 +3176,7 @@
     <t>Parameters.parameter</t>
   </si>
   <si>
-    <t>5</t>
+    <t>8</t>
   </si>
   <si>
     <t>Operation Parameter</t>
@@ -3341,6 +3341,97 @@
   </si>
   <si>
     <t>Parameters.parameter:matchResult.part</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchCreated</t>
+  </si>
+  <si>
+    <t>matchCreated</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchCreated.id</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchCreated.extension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchCreated.modifierExtension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchCreated.name</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchCreated.value[x]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dateTime
+</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchCreated.resource</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchCreated.part</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchCreationType</t>
+  </si>
+  <si>
+    <t>matchCreationType</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchCreationType.id</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchCreationType.extension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchCreationType.modifierExtension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchCreationType.name</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchCreationType.value[x]</t>
+  </si>
+  <si>
+    <t>https://ths-greifswald.de/fhir/epix/ValueSet/MatchCreationTypeVS</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchCreationType.resource</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchCreationType.part</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchPriority</t>
+  </si>
+  <si>
+    <t>matchPriority</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchPriority.id</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchPriority.extension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchPriority.modifierExtension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchPriority.name</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchPriority.value[x]</t>
+  </si>
+  <si>
+    <t>https://ths-greifswald.de/fhir/epix/ValueSet/MatchPriorityVS</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchPriority.resource</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchPriority.part</t>
   </si>
   <si>
     <t>Parameters.parameter:linkId</t>
@@ -4199,13 +4290,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK387"/>
+  <dimension ref="A1:AK411"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="21.71875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="60.3515625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="46.828125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="4" max="4" width="15.296875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="4" max="4" width="16.71484375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="34.8125" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="15.296875" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="4.21484375" customWidth="true" bestFit="true"/>
@@ -4221,14 +4312,14 @@
     <col min="17" max="17" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="19" max="19" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" width="10.95703125" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="16.71484375" customWidth="true" bestFit="true"/>
     <col min="21" max="21" width="34.80859375" customWidth="true" bestFit="true"/>
     <col min="22" max="22" width="14.08984375" customWidth="true" bestFit="true"/>
     <col min="23" max="23" width="14.4296875" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="15.31640625" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="14.62890625" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="88.69921875" customWidth="true" bestFit="true"/>
-    <col min="27" max="27" width="51.0234375" customWidth="true" bestFit="true"/>
+    <col min="27" max="27" width="55.16796875" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="5.10546875" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="17.6953125" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="35.90625" customWidth="true" bestFit="true"/>
@@ -44770,6 +44861,2510 @@
         <v>121</v>
       </c>
     </row>
+    <row r="388">
+      <c r="A388" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B388" t="s" s="2">
+        <v>1087</v>
+      </c>
+      <c r="C388" t="s" s="2">
+        <v>1022</v>
+      </c>
+      <c r="D388" t="s" s="2">
+        <v>1088</v>
+      </c>
+      <c r="E388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F388" s="2"/>
+      <c r="G388" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H388" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="I388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K388" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L388" t="s" s="2">
+        <v>722</v>
+      </c>
+      <c r="M388" t="s" s="2">
+        <v>1024</v>
+      </c>
+      <c r="N388" t="s" s="2">
+        <v>1025</v>
+      </c>
+      <c r="O388" s="2"/>
+      <c r="P388" s="2"/>
+      <c r="Q388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R388" s="2"/>
+      <c r="S388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG388" t="s" s="2">
+        <v>1022</v>
+      </c>
+      <c r="AH388" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI388" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ388" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK388" t="s" s="2">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B389" t="s" s="2">
+        <v>1089</v>
+      </c>
+      <c r="C389" t="s" s="2">
+        <v>1029</v>
+      </c>
+      <c r="D389" s="2"/>
+      <c r="E389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F389" s="2"/>
+      <c r="G389" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H389" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="I389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="L389" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="M389" t="s" s="2">
+        <v>86</v>
+      </c>
+      <c r="N389" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="O389" s="2"/>
+      <c r="P389" s="2"/>
+      <c r="Q389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R389" s="2"/>
+      <c r="S389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG389" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AH389" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI389" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AJ389" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK389" t="s" s="2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B390" t="s" s="2">
+        <v>1090</v>
+      </c>
+      <c r="C390" t="s" s="2">
+        <v>1030</v>
+      </c>
+      <c r="D390" s="2"/>
+      <c r="E390" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="F390" s="2"/>
+      <c r="G390" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H390" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="L390" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="M390" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="N390" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="O390" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="P390" s="2"/>
+      <c r="Q390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R390" s="2"/>
+      <c r="S390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG390" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="AH390" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI390" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ390" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK390" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B391" t="s" s="2">
+        <v>1091</v>
+      </c>
+      <c r="C391" t="s" s="2">
+        <v>1031</v>
+      </c>
+      <c r="D391" s="2"/>
+      <c r="E391" t="s" s="2">
+        <v>731</v>
+      </c>
+      <c r="F391" s="2"/>
+      <c r="G391" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H391" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J391" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="K391" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L391" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="M391" t="s" s="2">
+        <v>732</v>
+      </c>
+      <c r="N391" t="s" s="2">
+        <v>733</v>
+      </c>
+      <c r="O391" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="P391" t="s" s="2">
+        <v>466</v>
+      </c>
+      <c r="Q391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R391" s="2"/>
+      <c r="S391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG391" t="s" s="2">
+        <v>734</v>
+      </c>
+      <c r="AH391" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI391" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ391" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK391" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B392" t="s" s="2">
+        <v>1092</v>
+      </c>
+      <c r="C392" t="s" s="2">
+        <v>1032</v>
+      </c>
+      <c r="D392" s="2"/>
+      <c r="E392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F392" s="2"/>
+      <c r="G392" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H392" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="I392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K392" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L392" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="M392" t="s" s="2">
+        <v>1033</v>
+      </c>
+      <c r="N392" t="s" s="2">
+        <v>1034</v>
+      </c>
+      <c r="O392" s="2"/>
+      <c r="P392" s="2"/>
+      <c r="Q392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R392" s="2"/>
+      <c r="S392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T392" t="s" s="2">
+        <v>1088</v>
+      </c>
+      <c r="U392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG392" t="s" s="2">
+        <v>1032</v>
+      </c>
+      <c r="AH392" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI392" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AJ392" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK392" t="s" s="2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B393" t="s" s="2">
+        <v>1093</v>
+      </c>
+      <c r="C393" t="s" s="2">
+        <v>1035</v>
+      </c>
+      <c r="D393" s="2"/>
+      <c r="E393" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F393" s="2"/>
+      <c r="G393" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H393" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="I393" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J393" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K393" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L393" t="s" s="2">
+        <v>390</v>
+      </c>
+      <c r="M393" t="s" s="2">
+        <v>1036</v>
+      </c>
+      <c r="N393" t="s" s="2">
+        <v>1037</v>
+      </c>
+      <c r="O393" s="2"/>
+      <c r="P393" s="2"/>
+      <c r="Q393" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R393" s="2"/>
+      <c r="S393" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T393" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U393" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V393" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W393" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X393" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y393" t="s" s="2">
+        <v>304</v>
+      </c>
+      <c r="Z393" s="2"/>
+      <c r="AA393" t="s" s="2">
+        <v>1094</v>
+      </c>
+      <c r="AB393" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC393" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD393" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE393" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF393" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG393" t="s" s="2">
+        <v>1035</v>
+      </c>
+      <c r="AH393" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI393" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AJ393" t="s" s="2">
+        <v>1038</v>
+      </c>
+      <c r="AK393" t="s" s="2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B394" t="s" s="2">
+        <v>1095</v>
+      </c>
+      <c r="C394" t="s" s="2">
+        <v>1039</v>
+      </c>
+      <c r="D394" s="2"/>
+      <c r="E394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F394" s="2"/>
+      <c r="G394" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H394" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="I394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K394" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L394" t="s" s="2">
+        <v>271</v>
+      </c>
+      <c r="M394" t="s" s="2">
+        <v>1040</v>
+      </c>
+      <c r="N394" t="s" s="2">
+        <v>1041</v>
+      </c>
+      <c r="O394" t="s" s="2">
+        <v>1042</v>
+      </c>
+      <c r="P394" s="2"/>
+      <c r="Q394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R394" s="2"/>
+      <c r="S394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF394" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG394" t="s" s="2">
+        <v>1039</v>
+      </c>
+      <c r="AH394" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI394" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AJ394" t="s" s="2">
+        <v>1038</v>
+      </c>
+      <c r="AK394" t="s" s="2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B395" t="s" s="2">
+        <v>1096</v>
+      </c>
+      <c r="C395" t="s" s="2">
+        <v>1043</v>
+      </c>
+      <c r="D395" s="2"/>
+      <c r="E395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F395" s="2"/>
+      <c r="G395" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H395" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K395" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L395" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="M395" t="s" s="2">
+        <v>1044</v>
+      </c>
+      <c r="N395" t="s" s="2">
+        <v>1045</v>
+      </c>
+      <c r="O395" t="s" s="2">
+        <v>1046</v>
+      </c>
+      <c r="P395" s="2"/>
+      <c r="Q395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R395" s="2"/>
+      <c r="S395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG395" t="s" s="2">
+        <v>1043</v>
+      </c>
+      <c r="AH395" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI395" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ395" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK395" t="s" s="2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B396" t="s" s="2">
+        <v>1097</v>
+      </c>
+      <c r="C396" t="s" s="2">
+        <v>1022</v>
+      </c>
+      <c r="D396" t="s" s="2">
+        <v>1098</v>
+      </c>
+      <c r="E396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F396" s="2"/>
+      <c r="G396" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H396" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="I396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K396" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L396" t="s" s="2">
+        <v>722</v>
+      </c>
+      <c r="M396" t="s" s="2">
+        <v>1024</v>
+      </c>
+      <c r="N396" t="s" s="2">
+        <v>1025</v>
+      </c>
+      <c r="O396" s="2"/>
+      <c r="P396" s="2"/>
+      <c r="Q396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R396" s="2"/>
+      <c r="S396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG396" t="s" s="2">
+        <v>1022</v>
+      </c>
+      <c r="AH396" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI396" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ396" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK396" t="s" s="2">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B397" t="s" s="2">
+        <v>1099</v>
+      </c>
+      <c r="C397" t="s" s="2">
+        <v>1029</v>
+      </c>
+      <c r="D397" s="2"/>
+      <c r="E397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F397" s="2"/>
+      <c r="G397" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H397" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="I397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="L397" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="M397" t="s" s="2">
+        <v>86</v>
+      </c>
+      <c r="N397" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="O397" s="2"/>
+      <c r="P397" s="2"/>
+      <c r="Q397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R397" s="2"/>
+      <c r="S397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG397" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AH397" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI397" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AJ397" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK397" t="s" s="2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B398" t="s" s="2">
+        <v>1100</v>
+      </c>
+      <c r="C398" t="s" s="2">
+        <v>1030</v>
+      </c>
+      <c r="D398" s="2"/>
+      <c r="E398" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="F398" s="2"/>
+      <c r="G398" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H398" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="L398" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="M398" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="N398" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="O398" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="P398" s="2"/>
+      <c r="Q398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R398" s="2"/>
+      <c r="S398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG398" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="AH398" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI398" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ398" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK398" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B399" t="s" s="2">
+        <v>1101</v>
+      </c>
+      <c r="C399" t="s" s="2">
+        <v>1031</v>
+      </c>
+      <c r="D399" s="2"/>
+      <c r="E399" t="s" s="2">
+        <v>731</v>
+      </c>
+      <c r="F399" s="2"/>
+      <c r="G399" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H399" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J399" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="K399" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L399" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="M399" t="s" s="2">
+        <v>732</v>
+      </c>
+      <c r="N399" t="s" s="2">
+        <v>733</v>
+      </c>
+      <c r="O399" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="P399" t="s" s="2">
+        <v>466</v>
+      </c>
+      <c r="Q399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R399" s="2"/>
+      <c r="S399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG399" t="s" s="2">
+        <v>734</v>
+      </c>
+      <c r="AH399" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI399" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ399" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK399" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B400" t="s" s="2">
+        <v>1102</v>
+      </c>
+      <c r="C400" t="s" s="2">
+        <v>1032</v>
+      </c>
+      <c r="D400" s="2"/>
+      <c r="E400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F400" s="2"/>
+      <c r="G400" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H400" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="I400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K400" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L400" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="M400" t="s" s="2">
+        <v>1033</v>
+      </c>
+      <c r="N400" t="s" s="2">
+        <v>1034</v>
+      </c>
+      <c r="O400" s="2"/>
+      <c r="P400" s="2"/>
+      <c r="Q400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R400" s="2"/>
+      <c r="S400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T400" t="s" s="2">
+        <v>1098</v>
+      </c>
+      <c r="U400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG400" t="s" s="2">
+        <v>1032</v>
+      </c>
+      <c r="AH400" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI400" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AJ400" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK400" t="s" s="2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B401" t="s" s="2">
+        <v>1103</v>
+      </c>
+      <c r="C401" t="s" s="2">
+        <v>1035</v>
+      </c>
+      <c r="D401" s="2"/>
+      <c r="E401" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F401" s="2"/>
+      <c r="G401" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H401" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="I401" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J401" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K401" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L401" t="s" s="2">
+        <v>390</v>
+      </c>
+      <c r="M401" t="s" s="2">
+        <v>1036</v>
+      </c>
+      <c r="N401" t="s" s="2">
+        <v>1037</v>
+      </c>
+      <c r="O401" s="2"/>
+      <c r="P401" s="2"/>
+      <c r="Q401" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R401" s="2"/>
+      <c r="S401" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T401" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U401" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V401" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W401" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X401" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y401" t="s" s="2">
+        <v>304</v>
+      </c>
+      <c r="Z401" s="2"/>
+      <c r="AA401" t="s" s="2">
+        <v>1104</v>
+      </c>
+      <c r="AB401" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC401" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD401" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE401" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF401" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG401" t="s" s="2">
+        <v>1035</v>
+      </c>
+      <c r="AH401" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI401" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AJ401" t="s" s="2">
+        <v>1038</v>
+      </c>
+      <c r="AK401" t="s" s="2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B402" t="s" s="2">
+        <v>1105</v>
+      </c>
+      <c r="C402" t="s" s="2">
+        <v>1039</v>
+      </c>
+      <c r="D402" s="2"/>
+      <c r="E402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F402" s="2"/>
+      <c r="G402" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H402" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="I402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K402" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L402" t="s" s="2">
+        <v>271</v>
+      </c>
+      <c r="M402" t="s" s="2">
+        <v>1040</v>
+      </c>
+      <c r="N402" t="s" s="2">
+        <v>1041</v>
+      </c>
+      <c r="O402" t="s" s="2">
+        <v>1042</v>
+      </c>
+      <c r="P402" s="2"/>
+      <c r="Q402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R402" s="2"/>
+      <c r="S402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF402" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG402" t="s" s="2">
+        <v>1039</v>
+      </c>
+      <c r="AH402" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI402" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AJ402" t="s" s="2">
+        <v>1038</v>
+      </c>
+      <c r="AK402" t="s" s="2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B403" t="s" s="2">
+        <v>1106</v>
+      </c>
+      <c r="C403" t="s" s="2">
+        <v>1043</v>
+      </c>
+      <c r="D403" s="2"/>
+      <c r="E403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F403" s="2"/>
+      <c r="G403" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H403" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K403" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L403" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="M403" t="s" s="2">
+        <v>1044</v>
+      </c>
+      <c r="N403" t="s" s="2">
+        <v>1045</v>
+      </c>
+      <c r="O403" t="s" s="2">
+        <v>1046</v>
+      </c>
+      <c r="P403" s="2"/>
+      <c r="Q403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R403" s="2"/>
+      <c r="S403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG403" t="s" s="2">
+        <v>1043</v>
+      </c>
+      <c r="AH403" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI403" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ403" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK403" t="s" s="2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B404" t="s" s="2">
+        <v>1107</v>
+      </c>
+      <c r="C404" t="s" s="2">
+        <v>1022</v>
+      </c>
+      <c r="D404" t="s" s="2">
+        <v>1108</v>
+      </c>
+      <c r="E404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F404" s="2"/>
+      <c r="G404" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H404" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="I404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K404" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L404" t="s" s="2">
+        <v>722</v>
+      </c>
+      <c r="M404" t="s" s="2">
+        <v>1024</v>
+      </c>
+      <c r="N404" t="s" s="2">
+        <v>1025</v>
+      </c>
+      <c r="O404" s="2"/>
+      <c r="P404" s="2"/>
+      <c r="Q404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R404" s="2"/>
+      <c r="S404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG404" t="s" s="2">
+        <v>1022</v>
+      </c>
+      <c r="AH404" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI404" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ404" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK404" t="s" s="2">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B405" t="s" s="2">
+        <v>1109</v>
+      </c>
+      <c r="C405" t="s" s="2">
+        <v>1029</v>
+      </c>
+      <c r="D405" s="2"/>
+      <c r="E405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F405" s="2"/>
+      <c r="G405" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H405" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="I405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="L405" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="M405" t="s" s="2">
+        <v>86</v>
+      </c>
+      <c r="N405" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="O405" s="2"/>
+      <c r="P405" s="2"/>
+      <c r="Q405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R405" s="2"/>
+      <c r="S405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG405" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AH405" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI405" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AJ405" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK405" t="s" s="2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B406" t="s" s="2">
+        <v>1110</v>
+      </c>
+      <c r="C406" t="s" s="2">
+        <v>1030</v>
+      </c>
+      <c r="D406" s="2"/>
+      <c r="E406" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="F406" s="2"/>
+      <c r="G406" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H406" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="L406" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="M406" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="N406" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="O406" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="P406" s="2"/>
+      <c r="Q406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R406" s="2"/>
+      <c r="S406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG406" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="AH406" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI406" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ406" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK406" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B407" t="s" s="2">
+        <v>1111</v>
+      </c>
+      <c r="C407" t="s" s="2">
+        <v>1031</v>
+      </c>
+      <c r="D407" s="2"/>
+      <c r="E407" t="s" s="2">
+        <v>731</v>
+      </c>
+      <c r="F407" s="2"/>
+      <c r="G407" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H407" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J407" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="K407" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L407" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="M407" t="s" s="2">
+        <v>732</v>
+      </c>
+      <c r="N407" t="s" s="2">
+        <v>733</v>
+      </c>
+      <c r="O407" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="P407" t="s" s="2">
+        <v>466</v>
+      </c>
+      <c r="Q407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R407" s="2"/>
+      <c r="S407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG407" t="s" s="2">
+        <v>734</v>
+      </c>
+      <c r="AH407" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI407" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ407" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK407" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B408" t="s" s="2">
+        <v>1112</v>
+      </c>
+      <c r="C408" t="s" s="2">
+        <v>1032</v>
+      </c>
+      <c r="D408" s="2"/>
+      <c r="E408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F408" s="2"/>
+      <c r="G408" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H408" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="I408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K408" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L408" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="M408" t="s" s="2">
+        <v>1033</v>
+      </c>
+      <c r="N408" t="s" s="2">
+        <v>1034</v>
+      </c>
+      <c r="O408" s="2"/>
+      <c r="P408" s="2"/>
+      <c r="Q408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R408" s="2"/>
+      <c r="S408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T408" t="s" s="2">
+        <v>1108</v>
+      </c>
+      <c r="U408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG408" t="s" s="2">
+        <v>1032</v>
+      </c>
+      <c r="AH408" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI408" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AJ408" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK408" t="s" s="2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B409" t="s" s="2">
+        <v>1113</v>
+      </c>
+      <c r="C409" t="s" s="2">
+        <v>1035</v>
+      </c>
+      <c r="D409" s="2"/>
+      <c r="E409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F409" s="2"/>
+      <c r="G409" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H409" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="I409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K409" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L409" t="s" s="2">
+        <v>1114</v>
+      </c>
+      <c r="M409" t="s" s="2">
+        <v>1036</v>
+      </c>
+      <c r="N409" t="s" s="2">
+        <v>1037</v>
+      </c>
+      <c r="O409" s="2"/>
+      <c r="P409" s="2"/>
+      <c r="Q409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R409" s="2"/>
+      <c r="S409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF409" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG409" t="s" s="2">
+        <v>1035</v>
+      </c>
+      <c r="AH409" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI409" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AJ409" t="s" s="2">
+        <v>1038</v>
+      </c>
+      <c r="AK409" t="s" s="2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B410" t="s" s="2">
+        <v>1115</v>
+      </c>
+      <c r="C410" t="s" s="2">
+        <v>1039</v>
+      </c>
+      <c r="D410" s="2"/>
+      <c r="E410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F410" s="2"/>
+      <c r="G410" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H410" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="I410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K410" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L410" t="s" s="2">
+        <v>271</v>
+      </c>
+      <c r="M410" t="s" s="2">
+        <v>1040</v>
+      </c>
+      <c r="N410" t="s" s="2">
+        <v>1041</v>
+      </c>
+      <c r="O410" t="s" s="2">
+        <v>1042</v>
+      </c>
+      <c r="P410" s="2"/>
+      <c r="Q410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R410" s="2"/>
+      <c r="S410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF410" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG410" t="s" s="2">
+        <v>1039</v>
+      </c>
+      <c r="AH410" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI410" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AJ410" t="s" s="2">
+        <v>1038</v>
+      </c>
+      <c r="AK410" t="s" s="2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="s" s="2">
+        <v>1001</v>
+      </c>
+      <c r="B411" t="s" s="2">
+        <v>1116</v>
+      </c>
+      <c r="C411" t="s" s="2">
+        <v>1043</v>
+      </c>
+      <c r="D411" s="2"/>
+      <c r="E411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="F411" s="2"/>
+      <c r="G411" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H411" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="J411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="K411" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="L411" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="M411" t="s" s="2">
+        <v>1044</v>
+      </c>
+      <c r="N411" t="s" s="2">
+        <v>1045</v>
+      </c>
+      <c r="O411" t="s" s="2">
+        <v>1046</v>
+      </c>
+      <c r="P411" s="2"/>
+      <c r="Q411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="R411" s="2"/>
+      <c r="S411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="T411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="U411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="V411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="W411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="X411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Y411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="Z411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AA411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AB411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AD411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AE411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AF411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AG411" t="s" s="2">
+        <v>1043</v>
+      </c>
+      <c r="AH411" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI411" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ411" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="AK411" t="s" s="2">
+        <v>121</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
umarbeitung 2x addPossbileMatch für profile-MatchParameters.fsh
</commit_message>
<xml_diff>
--- a/output/all-profiles.xlsx
+++ b/output/all-profiles.xlsx
@@ -3407,35 +3407,35 @@
     <t>Parameters.parameter:matchPriority.part</t>
   </si>
   <si>
-    <t>Parameters.parameter:linkId</t>
-  </si>
-  <si>
-    <t>linkId</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:linkId.id</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:linkId.extension</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:linkId.modifierExtension</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:linkId.name</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:linkId.value[x]</t>
+    <t>Parameters.parameter:matchLinkId</t>
+  </si>
+  <si>
+    <t>matchLinkId</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchLinkId.id</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchLinkId.extension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchLinkId.modifierExtension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchLinkId.name</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchLinkId.value[x]</t>
   </si>
   <si>
     <t xml:space="preserve">integer
 </t>
   </si>
   <si>
-    <t>Parameters.parameter:linkId.resource</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:linkId.part</t>
+    <t>Parameters.parameter:matchLinkId.resource</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:matchLinkId.part</t>
   </si>
 </sst>
 </file>

</xml_diff>